<commit_message>
schema update to nightmarket table
</commit_message>
<xml_diff>
--- a/schema_v2.xlsx
+++ b/schema_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2abd1f54496c410b/Documents/GCP_test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="132" documentId="11_F25DC773A252ABDACC10481939DD4A0C5BDE58E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74367E3D-4D5A-4E9C-AFFE-DD5040DEF90D}"/>
+  <xr:revisionPtr revIDLastSave="133" documentId="11_F25DC773A252ABDACC10481939DD4A0C5BDE58E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8FF5609A-EE54-45EC-B67E-16E7EC32A06C}"/>
   <bookViews>
-    <workbookView xWindow="7760" yWindow="0" windowWidth="11530" windowHeight="12090" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
   <si>
     <t>accident_longitude</t>
   </si>
@@ -163,6 +163,10 @@
   <si>
     <t>A. sub_accident_history (歷史事故事件副表/fact)</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>city</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -662,6 +666,9 @@
       <c r="A10" s="4" t="s">
         <v>8</v>
       </c>
+      <c r="D10" s="4" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">

</xml_diff>